<commit_message>
Updated to allow for output to Excel and printing both scores/relevance
</commit_message>
<xml_diff>
--- a/test data.xlsx
+++ b/test data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tristanraffo/Downloads/code/Python/Senior Research/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{CFDD383B-36C6-754F-85A1-011BEDA77B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E86E11-4A98-794D-BA4F-65842C951417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16660" xr2:uid="{89450E28-0BB8-2040-BF54-F7AA5FA9F715}"/>
   </bookViews>
@@ -618,10 +618,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1033,7 +1032,7 @@
       <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" t="s">
         <v>27</v>
       </c>
       <c r="F2" t="str">
@@ -1052,10 +1051,10 @@
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" t="s">
         <v>26</v>
       </c>
       <c r="F3" t="str">
@@ -1084,7 +1083,7 @@
       <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" t="s">
         <v>24</v>
       </c>
       <c r="F4" t="str">
@@ -1108,7 +1107,7 @@
       <c r="D5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>23</v>
       </c>
       <c r="F5" t="str">
@@ -1135,7 +1134,7 @@
       <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>22</v>
       </c>
       <c r="F6" t="str">
@@ -1145,46 +1144,6 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B7" s="1"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E20" s="2"/>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B80" s="1"/>

</xml_diff>